<commit_message>
batch2 review sheet: google-fill the 13 obscure flora/fauna rows
</commit_message>
<xml_diff>
--- a/data/raw/override_batch2_review.xlsx
+++ b/data/raw/override_batch2_review.xlsx
@@ -502,7 +502,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -543,7 +542,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -584,7 +582,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -625,7 +622,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -666,7 +662,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -707,7 +702,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -748,7 +742,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -789,7 +782,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -830,7 +822,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -871,7 +862,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -912,7 +902,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -953,7 +942,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -994,7 +982,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1035,7 +1022,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1076,7 +1062,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1117,7 +1102,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1158,7 +1142,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1199,7 +1182,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1240,7 +1222,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1281,7 +1262,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1322,7 +1302,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1363,7 +1342,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1404,7 +1382,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1445,7 +1422,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1486,7 +1462,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1527,7 +1502,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1568,7 +1542,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1609,7 +1582,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1650,7 +1622,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1691,7 +1662,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1732,7 +1702,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1773,7 +1742,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1814,7 +1782,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1855,7 +1822,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1896,7 +1862,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1937,7 +1902,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1978,7 +1942,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2019,7 +1982,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2060,7 +2022,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2101,7 +2062,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2142,7 +2102,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2183,7 +2142,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2224,7 +2182,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2265,7 +2222,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2306,7 +2262,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2347,7 +2302,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2388,7 +2342,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2429,7 +2382,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2470,7 +2422,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2511,7 +2462,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2552,7 +2502,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2593,7 +2542,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2634,7 +2582,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2675,7 +2622,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2716,7 +2662,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2757,7 +2702,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2798,7 +2742,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2839,7 +2782,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2880,7 +2822,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2921,7 +2862,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2962,7 +2902,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3003,7 +2942,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3044,7 +2982,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3085,7 +3022,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3126,7 +3062,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3167,7 +3102,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3208,7 +3142,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3249,7 +3182,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3290,7 +3222,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3331,7 +3262,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3372,7 +3302,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3413,7 +3342,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3454,7 +3382,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3495,7 +3422,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3536,7 +3462,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -3577,7 +3502,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3618,7 +3542,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3659,7 +3582,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3700,7 +3622,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3741,7 +3662,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3782,7 +3702,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -3823,7 +3742,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -3864,7 +3782,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -3905,7 +3822,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -3946,7 +3862,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -3987,7 +3902,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -4028,7 +3942,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -4069,7 +3982,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -4090,8 +4002,16 @@
           <t>azelea</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
-      <c r="F90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>أزيليا</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>google-fallback</t>
+        </is>
+      </c>
       <c r="G90" t="inlineStr">
         <is>
           <t>untranslated-nonlatin</t>
@@ -4099,10 +4019,9 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>fill manually (no ref)</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr"/>
+          <t>obscure - low stakes, glance</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -4143,7 +4062,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -4164,8 +4082,16 @@
           <t>ginkgo</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
-      <c r="F92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>الجنكة</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>google-fallback</t>
+        </is>
+      </c>
       <c r="G92" t="inlineStr">
         <is>
           <t>untranslated-nonlatin</t>
@@ -4173,10 +4099,9 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>fill manually (no ref)</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr"/>
+          <t>obscure - low stakes, glance</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -4197,8 +4122,16 @@
           <t>gladiolus</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
-      <c r="F93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>الزنبق</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>google-fallback</t>
+        </is>
+      </c>
       <c r="G93" t="inlineStr">
         <is>
           <t>untranslated-nonlatin</t>
@@ -4206,10 +4139,9 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>fill manually (no ref)</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr"/>
+          <t>obscure - low stakes, glance</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -4250,7 +4182,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -4291,7 +4222,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -4312,8 +4242,16 @@
           <t>turtledove</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>حمامة السلحفاة</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>google-fallback</t>
+        </is>
+      </c>
       <c r="G96" t="inlineStr">
         <is>
           <t>untranslated-nonlatin</t>
@@ -4321,10 +4259,9 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>fill manually (no ref)</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr"/>
+          <t>obscure - low stakes, glance</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -4365,7 +4302,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -4386,8 +4322,16 @@
           <t>starfruit</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
-      <c r="F98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>כוכב ים</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>google-fallback</t>
+        </is>
+      </c>
       <c r="G98" t="inlineStr">
         <is>
           <t>untranslated-nonlatin</t>
@@ -4395,10 +4339,9 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>fill manually (no ref)</t>
-        </is>
-      </c>
-      <c r="I98" t="inlineStr"/>
+          <t>obscure - low stakes, glance</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -4419,8 +4362,16 @@
           <t>azalea</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Azalea</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>google-fallback</t>
+        </is>
+      </c>
       <c r="G99" t="inlineStr">
         <is>
           <t>untranslated-nonlatin</t>
@@ -4428,10 +4379,9 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>fill manually (no ref)</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr"/>
+          <t>obscure - low stakes, glance</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -4472,7 +4422,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -4513,7 +4462,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -4554,7 +4502,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -4595,7 +4542,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -4616,8 +4562,16 @@
           <t>elm</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
-      <c r="F104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>एल्म</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>google-fallback</t>
+        </is>
+      </c>
       <c r="G104" t="inlineStr">
         <is>
           <t>untranslated-nonlatin</t>
@@ -4625,10 +4579,9 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>fill manually (no ref)</t>
-        </is>
-      </c>
-      <c r="I104" t="inlineStr"/>
+          <t>obscure - low stakes, glance</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -4669,7 +4622,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -4690,8 +4642,16 @@
           <t>ginkgo</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
-      <c r="F106" t="inlineStr"/>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>जिन्कगो</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>google-fallback</t>
+        </is>
+      </c>
       <c r="G106" t="inlineStr">
         <is>
           <t>untranslated-nonlatin</t>
@@ -4699,10 +4659,9 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>fill manually (no ref)</t>
-        </is>
-      </c>
-      <c r="I106" t="inlineStr"/>
+          <t>obscure - low stakes, glance</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -4743,7 +4702,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -4784,7 +4742,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -4825,7 +4782,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -4846,8 +4802,16 @@
           <t>pelican</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
-      <c r="F110" t="inlineStr"/>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>हवासील</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>google-fallback</t>
+        </is>
+      </c>
       <c r="G110" t="inlineStr">
         <is>
           <t>untranslated-nonlatin</t>
@@ -4855,10 +4819,9 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>fill manually (no ref)</t>
-        </is>
-      </c>
-      <c r="I110" t="inlineStr"/>
+          <t>obscure - low stakes, glance</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -4899,7 +4862,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -4920,8 +4882,16 @@
           <t>seahorse</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
-      <c r="F112" t="inlineStr"/>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>समुद्री घोड़े</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>google-fallback</t>
+        </is>
+      </c>
       <c r="G112" t="inlineStr">
         <is>
           <t>untranslated-nonlatin</t>
@@ -4929,10 +4899,9 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>fill manually (no ref)</t>
-        </is>
-      </c>
-      <c r="I112" t="inlineStr"/>
+          <t>obscure - low stakes, glance</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -4973,7 +4942,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -5014,7 +4982,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -5055,7 +5022,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -5076,8 +5042,16 @@
           <t>stripe</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr"/>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>धारी</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>google-fallback</t>
+        </is>
+      </c>
       <c r="G116" t="inlineStr">
         <is>
           <t>untranslated-nonlatin</t>
@@ -5085,10 +5059,9 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>fill manually (no ref)</t>
-        </is>
-      </c>
-      <c r="I116" t="inlineStr"/>
+          <t>obscure - low stakes, glance</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -5129,7 +5102,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -5170,7 +5142,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -5191,8 +5162,16 @@
           <t>snapdragon</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
-      <c r="F119" t="inlineStr"/>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>キンギョソウ</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>google-fallback</t>
+        </is>
+      </c>
       <c r="G119" t="inlineStr">
         <is>
           <t>untranslated-nonlatin</t>
@@ -5200,10 +5179,9 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>fill manually (no ref)</t>
-        </is>
-      </c>
-      <c r="I119" t="inlineStr"/>
+          <t>obscure - low stakes, glance</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -5244,7 +5222,6 @@
           <t>from wiktionary - glance</t>
         </is>
       </c>
-      <c r="I120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -5265,8 +5242,16 @@
           <t>starfruit</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
-      <c r="F121" t="inlineStr"/>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>карамбола</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>google-fallback</t>
+        </is>
+      </c>
       <c r="G121" t="inlineStr">
         <is>
           <t>untranslated-nonlatin</t>
@@ -5274,10 +5259,9 @@
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>fill manually (no ref)</t>
-        </is>
-      </c>
-      <c r="I121" t="inlineStr"/>
+          <t>obscure - low stakes, glance</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -5313,8 +5297,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
-      <c r="I122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -5350,8 +5332,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
-      <c r="I123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -5387,8 +5367,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
-      <c r="I124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -5424,8 +5402,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
-      <c r="I125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -5461,8 +5437,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
-      <c r="I126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -5498,8 +5472,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
-      <c r="I127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -5535,8 +5507,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
-      <c r="I128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -5572,8 +5542,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
-      <c r="I129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -5609,8 +5577,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
-      <c r="I130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -5646,8 +5612,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
-      <c r="I131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -5683,8 +5647,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
-      <c r="I132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -5720,8 +5682,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
-      <c r="I133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -5757,8 +5717,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr"/>
-      <c r="I134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -5794,8 +5752,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H135" t="inlineStr"/>
-      <c r="I135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -5831,8 +5787,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H136" t="inlineStr"/>
-      <c r="I136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -5868,8 +5822,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr"/>
-      <c r="I137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -5905,8 +5857,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H138" t="inlineStr"/>
-      <c r="I138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -5942,8 +5892,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H139" t="inlineStr"/>
-      <c r="I139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -5979,8 +5927,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H140" t="inlineStr"/>
-      <c r="I140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -6016,8 +5962,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr"/>
-      <c r="I141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -6053,8 +5997,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H142" t="inlineStr"/>
-      <c r="I142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -6090,8 +6032,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H143" t="inlineStr"/>
-      <c r="I143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -6127,8 +6067,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H144" t="inlineStr"/>
-      <c r="I144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -6164,8 +6102,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr"/>
-      <c r="I145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -6201,8 +6137,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr"/>
-      <c r="I146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -6238,8 +6172,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H147" t="inlineStr"/>
-      <c r="I147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -6275,8 +6207,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr"/>
-      <c r="I148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -6312,8 +6242,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H149" t="inlineStr"/>
-      <c r="I149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -6349,8 +6277,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H150" t="inlineStr"/>
-      <c r="I150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -6386,8 +6312,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H151" t="inlineStr"/>
-      <c r="I151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -6423,8 +6347,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H152" t="inlineStr"/>
-      <c r="I152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -6460,8 +6382,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr"/>
-      <c r="I153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -6497,8 +6417,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H154" t="inlineStr"/>
-      <c r="I154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -6534,8 +6452,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H155" t="inlineStr"/>
-      <c r="I155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -6571,8 +6487,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H156" t="inlineStr"/>
-      <c r="I156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -6608,8 +6522,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H157" t="inlineStr"/>
-      <c r="I157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -6645,8 +6557,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H158" t="inlineStr"/>
-      <c r="I158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -6682,8 +6592,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H159" t="inlineStr"/>
-      <c r="I159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -6719,8 +6627,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H160" t="inlineStr"/>
-      <c r="I160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -6756,8 +6662,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H161" t="inlineStr"/>
-      <c r="I161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -6793,8 +6697,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H162" t="inlineStr"/>
-      <c r="I162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -6830,8 +6732,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H163" t="inlineStr"/>
-      <c r="I163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -6867,8 +6767,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H164" t="inlineStr"/>
-      <c r="I164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -6904,8 +6802,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H165" t="inlineStr"/>
-      <c r="I165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -6941,8 +6837,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H166" t="inlineStr"/>
-      <c r="I166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -6978,8 +6872,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H167" t="inlineStr"/>
-      <c r="I167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -7015,8 +6907,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H168" t="inlineStr"/>
-      <c r="I168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -7052,8 +6942,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H169" t="inlineStr"/>
-      <c r="I169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -7089,8 +6977,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H170" t="inlineStr"/>
-      <c r="I170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -7126,8 +7012,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H171" t="inlineStr"/>
-      <c r="I171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -7163,8 +7047,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H172" t="inlineStr"/>
-      <c r="I172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -7200,8 +7082,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H173" t="inlineStr"/>
-      <c r="I173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -7237,8 +7117,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr"/>
-      <c r="I174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -7274,8 +7152,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H175" t="inlineStr"/>
-      <c r="I175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -7311,8 +7187,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H176" t="inlineStr"/>
-      <c r="I176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -7348,8 +7222,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H177" t="inlineStr"/>
-      <c r="I177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -7385,8 +7257,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H178" t="inlineStr"/>
-      <c r="I178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -7422,8 +7292,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H179" t="inlineStr"/>
-      <c r="I179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -7459,8 +7327,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H180" t="inlineStr"/>
-      <c r="I180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -7496,8 +7362,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H181" t="inlineStr"/>
-      <c r="I181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -7533,8 +7397,6 @@
           <t>greek-na-verb</t>
         </is>
       </c>
-      <c r="H182" t="inlineStr"/>
-      <c r="I182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -7570,8 +7432,6 @@
           <t>homoglyph</t>
         </is>
       </c>
-      <c r="H183" t="inlineStr"/>
-      <c r="I183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -7607,8 +7467,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H184" t="inlineStr"/>
-      <c r="I184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -7644,8 +7502,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H185" t="inlineStr"/>
-      <c r="I185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -7681,8 +7537,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H186" t="inlineStr"/>
-      <c r="I186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -7718,8 +7572,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H187" t="inlineStr"/>
-      <c r="I187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -7755,8 +7607,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H188" t="inlineStr"/>
-      <c r="I188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -7792,8 +7642,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H189" t="inlineStr"/>
-      <c r="I189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -7829,8 +7677,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H190" t="inlineStr"/>
-      <c r="I190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -7866,8 +7712,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H191" t="inlineStr"/>
-      <c r="I191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -7903,8 +7747,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H192" t="inlineStr"/>
-      <c r="I192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -7940,8 +7782,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H193" t="inlineStr"/>
-      <c r="I193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -7977,8 +7817,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H194" t="inlineStr"/>
-      <c r="I194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -8014,8 +7852,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H195" t="inlineStr"/>
-      <c r="I195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -8051,8 +7887,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H196" t="inlineStr"/>
-      <c r="I196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -8088,8 +7922,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H197" t="inlineStr"/>
-      <c r="I197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -8125,8 +7957,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H198" t="inlineStr"/>
-      <c r="I198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -8162,8 +7992,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H199" t="inlineStr"/>
-      <c r="I199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -8199,8 +8027,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H200" t="inlineStr"/>
-      <c r="I200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -8236,8 +8062,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H201" t="inlineStr"/>
-      <c r="I201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -8273,8 +8097,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H202" t="inlineStr"/>
-      <c r="I202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -8310,8 +8132,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H203" t="inlineStr"/>
-      <c r="I203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -8347,8 +8167,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H204" t="inlineStr"/>
-      <c r="I204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -8384,8 +8202,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H205" t="inlineStr"/>
-      <c r="I205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -8421,8 +8237,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H206" t="inlineStr"/>
-      <c r="I206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -8458,8 +8272,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H207" t="inlineStr"/>
-      <c r="I207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -8495,8 +8307,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H208" t="inlineStr"/>
-      <c r="I208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -8532,8 +8342,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H209" t="inlineStr"/>
-      <c r="I209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -8569,8 +8377,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H210" t="inlineStr"/>
-      <c r="I210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -8606,8 +8412,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H211" t="inlineStr"/>
-      <c r="I211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -8643,8 +8447,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H212" t="inlineStr"/>
-      <c r="I212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -8680,8 +8482,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H213" t="inlineStr"/>
-      <c r="I213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -8717,8 +8517,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H214" t="inlineStr"/>
-      <c r="I214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -8754,8 +8552,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H215" t="inlineStr"/>
-      <c r="I215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -8791,8 +8587,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H216" t="inlineStr"/>
-      <c r="I216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -8828,8 +8622,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H217" t="inlineStr"/>
-      <c r="I217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -8865,8 +8657,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H218" t="inlineStr"/>
-      <c r="I218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -8902,8 +8692,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H219" t="inlineStr"/>
-      <c r="I219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -8939,8 +8727,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H220" t="inlineStr"/>
-      <c r="I220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -8976,8 +8762,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H221" t="inlineStr"/>
-      <c r="I221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -9013,8 +8797,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H222" t="inlineStr"/>
-      <c r="I222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -9050,8 +8832,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H223" t="inlineStr"/>
-      <c r="I223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -9087,8 +8867,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H224" t="inlineStr"/>
-      <c r="I224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -9124,8 +8902,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H225" t="inlineStr"/>
-      <c r="I225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -9161,8 +8937,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H226" t="inlineStr"/>
-      <c r="I226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -9198,8 +8972,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr"/>
-      <c r="I227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -9235,8 +9007,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H228" t="inlineStr"/>
-      <c r="I228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -9272,8 +9042,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H229" t="inlineStr"/>
-      <c r="I229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -9309,8 +9077,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H230" t="inlineStr"/>
-      <c r="I230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -9346,8 +9112,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H231" t="inlineStr"/>
-      <c r="I231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -9383,8 +9147,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H232" t="inlineStr"/>
-      <c r="I232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -9420,8 +9182,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H233" t="inlineStr"/>
-      <c r="I233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -9457,8 +9217,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H234" t="inlineStr"/>
-      <c r="I234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -9494,8 +9252,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H235" t="inlineStr"/>
-      <c r="I235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -9531,8 +9287,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H236" t="inlineStr"/>
-      <c r="I236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -9568,8 +9322,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H237" t="inlineStr"/>
-      <c r="I237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -9605,8 +9357,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H238" t="inlineStr"/>
-      <c r="I238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -9642,8 +9392,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H239" t="inlineStr"/>
-      <c r="I239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -9679,8 +9427,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H240" t="inlineStr"/>
-      <c r="I240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -9716,8 +9462,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H241" t="inlineStr"/>
-      <c r="I241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -9753,8 +9497,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H242" t="inlineStr"/>
-      <c r="I242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -9790,8 +9532,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H243" t="inlineStr"/>
-      <c r="I243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -9827,8 +9567,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H244" t="inlineStr"/>
-      <c r="I244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -9864,8 +9602,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H245" t="inlineStr"/>
-      <c r="I245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -9901,8 +9637,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H246" t="inlineStr"/>
-      <c r="I246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -9938,8 +9672,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H247" t="inlineStr"/>
-      <c r="I247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -9975,8 +9707,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H248" t="inlineStr"/>
-      <c r="I248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -10012,8 +9742,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H249" t="inlineStr"/>
-      <c r="I249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -10049,8 +9777,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H250" t="inlineStr"/>
-      <c r="I250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -10086,8 +9812,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H251" t="inlineStr"/>
-      <c r="I251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -10123,8 +9847,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H252" t="inlineStr"/>
-      <c r="I252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -10160,8 +9882,6 @@
           <t>korean-sentence</t>
         </is>
       </c>
-      <c r="H253" t="inlineStr"/>
-      <c r="I253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -10197,8 +9917,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H254" t="inlineStr"/>
-      <c r="I254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -10234,8 +9952,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H255" t="inlineStr"/>
-      <c r="I255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -10271,8 +9987,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H256" t="inlineStr"/>
-      <c r="I256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -10308,8 +10022,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H257" t="inlineStr"/>
-      <c r="I257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -10345,8 +10057,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H258" t="inlineStr"/>
-      <c r="I258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -10382,8 +10092,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H259" t="inlineStr"/>
-      <c r="I259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -10419,8 +10127,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H260" t="inlineStr"/>
-      <c r="I260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -10456,8 +10162,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H261" t="inlineStr"/>
-      <c r="I261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -10493,8 +10197,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H262" t="inlineStr"/>
-      <c r="I262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -10530,8 +10232,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H263" t="inlineStr"/>
-      <c r="I263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -10567,8 +10267,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H264" t="inlineStr"/>
-      <c r="I264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -10604,8 +10302,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H265" t="inlineStr"/>
-      <c r="I265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -10641,8 +10337,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H266" t="inlineStr"/>
-      <c r="I266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -10678,8 +10372,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H267" t="inlineStr"/>
-      <c r="I267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -10715,8 +10407,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H268" t="inlineStr"/>
-      <c r="I268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -10752,8 +10442,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H269" t="inlineStr"/>
-      <c r="I269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -10789,8 +10477,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H270" t="inlineStr"/>
-      <c r="I270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -10826,8 +10512,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H271" t="inlineStr"/>
-      <c r="I271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -10863,8 +10547,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H272" t="inlineStr"/>
-      <c r="I272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -10900,8 +10582,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H273" t="inlineStr"/>
-      <c r="I273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -10937,8 +10617,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H274" t="inlineStr"/>
-      <c r="I274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -10974,8 +10652,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H275" t="inlineStr"/>
-      <c r="I275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -11011,8 +10687,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H276" t="inlineStr"/>
-      <c r="I276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="n">
@@ -11048,8 +10722,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H277" t="inlineStr"/>
-      <c r="I277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="n">
@@ -11085,8 +10757,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H278" t="inlineStr"/>
-      <c r="I278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="n">
@@ -11122,8 +10792,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H279" t="inlineStr"/>
-      <c r="I279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="n">
@@ -11159,8 +10827,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H280" t="inlineStr"/>
-      <c r="I280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="n">
@@ -11196,8 +10862,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H281" t="inlineStr"/>
-      <c r="I281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="n">
@@ -11233,8 +10897,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H282" t="inlineStr"/>
-      <c r="I282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="n">
@@ -11270,8 +10932,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H283" t="inlineStr"/>
-      <c r="I283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="n">
@@ -11307,8 +10967,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H284" t="inlineStr"/>
-      <c r="I284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="n">
@@ -11344,8 +11002,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H285" t="inlineStr"/>
-      <c r="I285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="n">
@@ -11381,8 +11037,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H286" t="inlineStr"/>
-      <c r="I286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="n">
@@ -11418,8 +11072,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H287" t="inlineStr"/>
-      <c r="I287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="n">
@@ -11455,8 +11107,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H288" t="inlineStr"/>
-      <c r="I288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="n">
@@ -11492,8 +11142,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H289" t="inlineStr"/>
-      <c r="I289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="n">
@@ -11529,8 +11177,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H290" t="inlineStr"/>
-      <c r="I290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="n">
@@ -11566,8 +11212,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H291" t="inlineStr"/>
-      <c r="I291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="n">
@@ -11603,8 +11247,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H292" t="inlineStr"/>
-      <c r="I292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="n">
@@ -11640,8 +11282,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H293" t="inlineStr"/>
-      <c r="I293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="n">
@@ -11677,8 +11317,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H294" t="inlineStr"/>
-      <c r="I294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="n">
@@ -11714,8 +11352,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H295" t="inlineStr"/>
-      <c r="I295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="n">
@@ -11751,8 +11387,6 @@
           <t>untranslated-differ-both</t>
         </is>
       </c>
-      <c r="H296" t="inlineStr"/>
-      <c r="I296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="n">
@@ -11788,8 +11422,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H297" t="inlineStr"/>
-      <c r="I297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="n">
@@ -11825,8 +11457,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H298" t="inlineStr"/>
-      <c r="I298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="n">
@@ -11862,8 +11492,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H299" t="inlineStr"/>
-      <c r="I299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="n">
@@ -11899,8 +11527,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H300" t="inlineStr"/>
-      <c r="I300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="n">
@@ -11936,8 +11562,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H301" t="inlineStr"/>
-      <c r="I301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="n">
@@ -11973,8 +11597,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H302" t="inlineStr"/>
-      <c r="I302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="n">
@@ -12010,8 +11632,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H303" t="inlineStr"/>
-      <c r="I303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="n">
@@ -12047,8 +11667,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H304" t="inlineStr"/>
-      <c r="I304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="n">
@@ -12084,8 +11702,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H305" t="inlineStr"/>
-      <c r="I305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="n">
@@ -12121,8 +11737,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H306" t="inlineStr"/>
-      <c r="I306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="n">
@@ -12158,8 +11772,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H307" t="inlineStr"/>
-      <c r="I307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="n">
@@ -12195,8 +11807,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H308" t="inlineStr"/>
-      <c r="I308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="n">
@@ -12232,8 +11842,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H309" t="inlineStr"/>
-      <c r="I309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="n">
@@ -12269,8 +11877,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H310" t="inlineStr"/>
-      <c r="I310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="n">
@@ -12306,8 +11912,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H311" t="inlineStr"/>
-      <c r="I311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="n">
@@ -12343,8 +11947,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H312" t="inlineStr"/>
-      <c r="I312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="n">
@@ -12380,8 +11982,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H313" t="inlineStr"/>
-      <c r="I313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="n">
@@ -12417,8 +12017,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H314" t="inlineStr"/>
-      <c r="I314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="n">
@@ -12454,8 +12052,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H315" t="inlineStr"/>
-      <c r="I315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="n">
@@ -12491,8 +12087,6 @@
           <t>untranslated-nonlatin</t>
         </is>
       </c>
-      <c r="H316" t="inlineStr"/>
-      <c r="I316" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>